<commit_message>
`Updated code with various changes across multiple files`
</commit_message>
<xml_diff>
--- a/SupportFiles/tool_list.xlsx
+++ b/SupportFiles/tool_list.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Ishan\Startups\Tool_Costing\SupportFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D62C299-AEAB-441C-950E-DB5B6E423A66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AC1BA7B-E135-4597-BF66-B0A80EAA542A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="24" yWindow="24" windowWidth="23016" windowHeight="12216" xr2:uid="{0EFB6794-C011-455C-9CA2-96EBF70FD493}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
   <si>
     <t>No</t>
   </si>
@@ -36,47 +36,119 @@
     <t>Part_Desc</t>
   </si>
   <si>
-    <t>ABC000</t>
-  </si>
-  <si>
-    <t>ABC111</t>
-  </si>
-  <si>
-    <t>ABC222</t>
-  </si>
-  <si>
-    <t>ABC333</t>
-  </si>
-  <si>
-    <t>ABC444</t>
-  </si>
-  <si>
-    <t>This is 1st Part</t>
-  </si>
-  <si>
-    <t>This is 2nd Part</t>
-  </si>
-  <si>
-    <t>This is 3rd Part</t>
-  </si>
-  <si>
-    <t>This is 4th Part</t>
-  </si>
-  <si>
-    <t>This is 5th Part</t>
-  </si>
-  <si>
     <t>Qty</t>
+  </si>
+  <si>
+    <t>Unit_Price</t>
+  </si>
+  <si>
+    <t>Total_Price</t>
+  </si>
+  <si>
+    <t>23-02322-0909-890-A-001-0002</t>
+  </si>
+  <si>
+    <t>23-02322-0909-890-A-001-0001</t>
+  </si>
+  <si>
+    <t>23-02322-0909-890-A-001-0003</t>
+  </si>
+  <si>
+    <t>23-02322-0909-890-A-001-0004</t>
+  </si>
+  <si>
+    <t>23-02322-0909-890-A-001-0005</t>
+  </si>
+  <si>
+    <t>23-02322-0909-890-A-001-0006</t>
+  </si>
+  <si>
+    <t>23-02322-0909-890-A-001-0007</t>
+  </si>
+  <si>
+    <t>23-02322-0909-890-A-001-0008</t>
+  </si>
+  <si>
+    <t>23-02322-0909-890-A-001-0009</t>
+  </si>
+  <si>
+    <t>23-02322-0909-890-A-001-0010</t>
+  </si>
+  <si>
+    <t>23-02322-0909-890-A-001-0011</t>
+  </si>
+  <si>
+    <t>23-02322-0909-890-A-001-0012</t>
+  </si>
+  <si>
+    <t>23-02322-0909-890-A-001-0013</t>
+  </si>
+  <si>
+    <t>23-02322-0909-890-A-001-0014</t>
+  </si>
+  <si>
+    <t>23-02322-0909-890-A-001-0015</t>
+  </si>
+  <si>
+    <t>Part 1</t>
+  </si>
+  <si>
+    <t>Part 2</t>
+  </si>
+  <si>
+    <t>Part 3</t>
+  </si>
+  <si>
+    <t>Part 4</t>
+  </si>
+  <si>
+    <t>Part 5</t>
+  </si>
+  <si>
+    <t>Part 6</t>
+  </si>
+  <si>
+    <t>Part 7</t>
+  </si>
+  <si>
+    <t>Part 8</t>
+  </si>
+  <si>
+    <t>Part 9</t>
+  </si>
+  <si>
+    <t>Part 10</t>
+  </si>
+  <si>
+    <t>Part 11</t>
+  </si>
+  <si>
+    <t>Part 12</t>
+  </si>
+  <si>
+    <t>Part 13</t>
+  </si>
+  <si>
+    <t>Part 14</t>
+  </si>
+  <si>
+    <t>Part 15</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -418,15 +490,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63236AF8-F01C-43FC-9B8F-7ACF1897A446}">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="6.21875" customWidth="1"/>
-    <col min="2" max="2" width="11.6640625" customWidth="1"/>
+    <col min="2" max="2" width="54.44140625" customWidth="1"/>
     <col min="3" max="3" width="21.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -437,80 +509,332 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D2">
+        <v>2</v>
+      </c>
+      <c r="E2">
+        <v>900</v>
+      </c>
+      <c r="F2">
+        <f>D2*E2</f>
+        <v>1800</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D3">
         <v>3</v>
       </c>
-      <c r="C2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E3">
+        <v>800</v>
+      </c>
+      <c r="F3">
+        <f t="shared" ref="F3:F16" si="0">D3*E3</f>
+        <v>2400</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C4" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="D4">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+        <v>2</v>
+      </c>
+      <c r="E4">
+        <v>750</v>
+      </c>
+      <c r="F4">
+        <f t="shared" si="0"/>
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C5" t="s">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="D5">
         <v>4</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E5">
+        <v>540</v>
+      </c>
+      <c r="F5">
+        <f t="shared" si="0"/>
+        <v>2160</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" t="s">
+        <v>25</v>
+      </c>
+      <c r="D6">
+        <v>2</v>
+      </c>
+      <c r="E6">
+        <v>300</v>
+      </c>
+      <c r="F6">
+        <f t="shared" si="0"/>
+        <v>600</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7" t="s">
+        <v>26</v>
+      </c>
+      <c r="D7">
+        <v>3</v>
+      </c>
+      <c r="E7">
+        <v>900</v>
+      </c>
+      <c r="F7">
+        <f t="shared" si="0"/>
+        <v>2700</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8">
         <v>7</v>
       </c>
-      <c r="C6" t="s">
+      <c r="B8" t="s">
         <v>12</v>
       </c>
-      <c r="D6">
-        <v>5</v>
+      <c r="C8" t="s">
+        <v>27</v>
+      </c>
+      <c r="D8">
+        <v>2</v>
+      </c>
+      <c r="E8">
+        <v>800</v>
+      </c>
+      <c r="F8">
+        <f t="shared" si="0"/>
+        <v>1600</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>13</v>
+      </c>
+      <c r="C9" t="s">
+        <v>28</v>
+      </c>
+      <c r="D9">
+        <v>4</v>
+      </c>
+      <c r="E9">
+        <v>750</v>
+      </c>
+      <c r="F9">
+        <f t="shared" si="0"/>
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C10" t="s">
+        <v>29</v>
+      </c>
+      <c r="D10">
+        <v>2</v>
+      </c>
+      <c r="E10">
+        <v>540</v>
+      </c>
+      <c r="F10">
+        <f t="shared" si="0"/>
+        <v>1080</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>15</v>
+      </c>
+      <c r="C11" t="s">
+        <v>30</v>
+      </c>
+      <c r="D11">
+        <v>3</v>
+      </c>
+      <c r="E11">
+        <v>300</v>
+      </c>
+      <c r="F11">
+        <f t="shared" si="0"/>
+        <v>900</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>16</v>
+      </c>
+      <c r="C12" t="s">
+        <v>31</v>
+      </c>
+      <c r="D12">
+        <v>2</v>
+      </c>
+      <c r="E12">
+        <v>900</v>
+      </c>
+      <c r="F12">
+        <f t="shared" si="0"/>
+        <v>1800</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>17</v>
+      </c>
+      <c r="C13" t="s">
+        <v>32</v>
+      </c>
+      <c r="D13">
+        <v>4</v>
+      </c>
+      <c r="E13">
+        <v>800</v>
+      </c>
+      <c r="F13">
+        <f t="shared" si="0"/>
+        <v>3200</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>18</v>
+      </c>
+      <c r="C14" t="s">
+        <v>33</v>
+      </c>
+      <c r="D14">
+        <v>2</v>
+      </c>
+      <c r="E14">
+        <v>750</v>
+      </c>
+      <c r="F14">
+        <f t="shared" si="0"/>
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>19</v>
+      </c>
+      <c r="C15" t="s">
+        <v>34</v>
+      </c>
+      <c r="D15">
+        <v>3</v>
+      </c>
+      <c r="E15">
+        <v>540</v>
+      </c>
+      <c r="F15">
+        <f t="shared" si="0"/>
+        <v>1620</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
+        <v>20</v>
+      </c>
+      <c r="C16" t="s">
+        <v>35</v>
+      </c>
+      <c r="D16">
+        <v>2</v>
+      </c>
+      <c r="E16">
+        <v>300</v>
+      </c>
+      <c r="F16">
+        <f t="shared" si="0"/>
+        <v>600</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>